<commit_message>
feat: complete EAM and payment workflow updates
</commit_message>
<xml_diff>
--- a/backend/yudao-module-eam/src/main/resources/eam/eam-asset-ledger-template.xlsx
+++ b/backend/yudao-module-eam/src/main/resources/eam/eam-asset-ledger-template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产台账" sheetId="1" r:id="R0cbc21e325bb426b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类字段说明" sheetId="2" r:id="Rc1c23588d30e49b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字典选项" sheetId="3" r:id="R51d5854f84ad4313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="4" r:id="R2a7a5b9e16db4d26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="资产台账" sheetId="1" r:id="Ra434e6e22527487a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类字段说明" sheetId="2" r:id="R74eb2c6e0c694b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字典选项" sheetId="3" r:id="R5e75916932c84e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="4" r:id="R61b25c64deb9407a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -351,161 +351,147 @@
         <x:v>资产状态</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>品牌型号</x:v>
+        <x:v>购入日期</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>规格参数</x:v>
+        <x:v>资产来源</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>序列号</x:v>
+        <x:v>使用人</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>条码</x:v>
+        <x:v>存放地点</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>原值</x:v>
+        <x:v>备注</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>净值</x:v>
+        <x:v>sn:序列号</x:v>
       </x:c>
       <x:c r="L1" s="4" t="str">
-        <x:v>购入日期</x:v>
+        <x:v>device_model:机型</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>资产来源</x:v>
+        <x:v>cpu:CPU</x:v>
       </x:c>
       <x:c r="N1" s="4" t="str">
-        <x:v>保修到期日</x:v>
+        <x:v>memory:内存</x:v>
       </x:c>
       <x:c r="O1" s="3" t="str">
-        <x:v>使用人</x:v>
+        <x:v>disk:硬盘</x:v>
       </x:c>
       <x:c r="P1" s="3" t="str">
-        <x:v>存放地点</x:v>
+        <x:v>color:外观颜色</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="str">
-        <x:v>预计使用年限（月）</x:v>
+        <x:v>power_adapter:电源适配器</x:v>
       </x:c>
       <x:c r="R1" s="3" t="str">
-        <x:v>备注</x:v>
+        <x:v>cables:配套线材</x:v>
       </x:c>
       <x:c r="S1" s="3" t="str">
-        <x:v>device_model:机型</x:v>
+        <x:v>original_box:原装包装盒</x:v>
       </x:c>
       <x:c r="T1" s="3" t="str">
-        <x:v>cpu:CPU</x:v>
+        <x:v>device_type:设备类型</x:v>
       </x:c>
       <x:c r="U1" s="3" t="str">
-        <x:v>memory:内存</x:v>
+        <x:v>mobile_system:手机系统</x:v>
       </x:c>
       <x:c r="V1" s="3" t="str">
-        <x:v>disk:硬盘</x:v>
+        <x:v>storage_capacity:存储容量</x:v>
       </x:c>
       <x:c r="W1" s="3" t="str">
-        <x:v>color:外观颜色</x:v>
+        <x:v>purpose:用途</x:v>
       </x:c>
       <x:c r="X1" s="3" t="str">
-        <x:v>power_adapter:电源适配器</x:v>
+        <x:v>display_size_resolution:尺寸/分辨率</x:v>
       </x:c>
       <x:c r="Y1" s="3" t="str">
-        <x:v>cables:配套线材</x:v>
+        <x:v>specification:规格/型号</x:v>
       </x:c>
       <x:c r="Z1" s="3" t="str">
-        <x:v>original_box:原装包装盒</x:v>
+        <x:v>login_id:登录账号/ID</x:v>
       </x:c>
       <x:c r="AA1" s="3" t="str">
-        <x:v>device_type:设备类型</x:v>
+        <x:v>account_name:账号名称</x:v>
       </x:c>
       <x:c r="AB1" s="3" t="str">
-        <x:v>mobile_system:手机系统</x:v>
+        <x:v>bound_mobile:绑定手机号</x:v>
       </x:c>
       <x:c r="AC1" s="3" t="str">
-        <x:v>storage_capacity:存储容量</x:v>
+        <x:v>password_custody:密码保管方式</x:v>
       </x:c>
       <x:c r="AD1" s="3" t="str">
-        <x:v>purpose:用途</x:v>
+        <x:v>platform:所属平台</x:v>
       </x:c>
       <x:c r="AE1" s="3" t="str">
-        <x:v>display_size_resolution:尺寸/分辨率</x:v>
+        <x:v>account_nature:账号性质</x:v>
       </x:c>
       <x:c r="AF1" s="3" t="str">
-        <x:v>specification:规格/型号</x:v>
+        <x:v>real_name_person:实名认证人</x:v>
       </x:c>
       <x:c r="AG1" s="3" t="str">
-        <x:v>login_id:登录账号/ID</x:v>
+        <x:v>bound_wechat_qq:绑定微信/QQ</x:v>
       </x:c>
       <x:c r="AH1" s="3" t="str">
-        <x:v>account_name:账号名称</x:v>
+        <x:v>contact_count:联系人数</x:v>
       </x:c>
       <x:c r="AI1" s="3" t="str">
-        <x:v>bound_mobile:绑定手机号</x:v>
+        <x:v>service_type:服务类型</x:v>
       </x:c>
       <x:c r="AJ1" s="3" t="str">
-        <x:v>password_custody:密码保管方式</x:v>
+        <x:v>service_name:服务名称</x:v>
       </x:c>
       <x:c r="AK1" s="3" t="str">
-        <x:v>platform:所属平台</x:v>
+        <x:v>membership_level:会员/套餐等级</x:v>
       </x:c>
       <x:c r="AL1" s="3" t="str">
-        <x:v>account_nature:账号性质</x:v>
+        <x:v>package_expiry:套餐到期日</x:v>
       </x:c>
       <x:c r="AM1" s="3" t="str">
-        <x:v>real_name_person:实名认证人</x:v>
+        <x:v>auto_renewal:是否自动续费</x:v>
       </x:c>
       <x:c r="AN1" s="3" t="str">
-        <x:v>bound_wechat_qq:绑定微信/QQ</x:v>
+        <x:v>payment_method:付费方式</x:v>
       </x:c>
       <x:c r="AO1" s="3" t="str">
-        <x:v>contact_count:联系人数</x:v>
+        <x:v>account_balance:账户当前余额</x:v>
       </x:c>
       <x:c r="AP1" s="3" t="str">
-        <x:v>service_type:服务类型</x:v>
+        <x:v>material:材质</x:v>
       </x:c>
       <x:c r="AQ1" s="3" t="str">
-        <x:v>service_name:服务名称</x:v>
+        <x:v>furniture_type:类型</x:v>
       </x:c>
       <x:c r="AR1" s="3" t="str">
-        <x:v>membership_level:会员/套餐等级</x:v>
+        <x:v>subject:所属科目</x:v>
       </x:c>
       <x:c r="AS1" s="3" t="str">
-        <x:v>package_expiry:套餐到期日</x:v>
+        <x:v>publisher:出版社</x:v>
       </x:c>
       <x:c r="AT1" s="3" t="str">
-        <x:v>auto_renewal:是否自动续费</x:v>
+        <x:v>author:作者</x:v>
       </x:c>
       <x:c r="AU1" s="3" t="str">
-        <x:v>payment_method:付费方式</x:v>
+        <x:v>isbn:ISBN</x:v>
       </x:c>
       <x:c r="AV1" s="3" t="str">
-        <x:v>account_balance:账户当前余额</x:v>
+        <x:v>edition_year:版次/年份</x:v>
       </x:c>
       <x:c r="AW1" s="3" t="str">
-        <x:v>material:材质</x:v>
+        <x:v>price:定价（元）</x:v>
       </x:c>
       <x:c r="AX1" s="3" t="str">
-        <x:v>furniture_type:类型</x:v>
-      </x:c>
-      <x:c r="AY1" s="3" t="str">
-        <x:v>subject:所属科目</x:v>
-      </x:c>
-      <x:c r="AZ1" s="3" t="str">
-        <x:v>publisher:出版社</x:v>
-      </x:c>
-      <x:c r="BA1" s="3" t="str">
-        <x:v>author:作者</x:v>
-      </x:c>
-      <x:c r="BB1" s="3" t="str">
-        <x:v>isbn:ISBN</x:v>
-      </x:c>
-      <x:c r="BC1" s="3" t="str">
-        <x:v>edition_year:版次/年份</x:v>
-      </x:c>
-      <x:c r="BD1" s="3" t="str">
-        <x:v>price:定价（元）</x:v>
-      </x:c>
-      <x:c r="BE1" s="3" t="str">
         <x:v>size:规格尺寸</x:v>
       </x:c>
+      <x:c r="AY1" s="3"/>
+      <x:c r="AZ1" s="3"/>
+      <x:c r="BA1" s="3"/>
+      <x:c r="BB1" s="3"/>
+      <x:c r="BC1" s="3"/>
+      <x:c r="BD1" s="3"/>
+      <x:c r="BE1" s="3"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2"/>
@@ -1979,6 +1965,27 @@
       <x:c r="F71" t="str"/>
       <x:c r="G71" t="str"/>
     </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>IT</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>IT硬件设备</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>sn</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>序列号</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>单行文本</x:v>
+      </x:c>
+      <x:c r="F72"/>
+      <x:c r="G72" t="str">
+        <x:v>由 IT 根分类继承至全部子分类，选填</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2164,6 +2171,11 @@
         <x:v>7. 日期统一使用 yyyy-mm-dd。</x:v>
       </x:c>
     </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>序列号使用 sn:序列号 自定义列，仅适用于已配置该字段的 IT 分类。品牌型号等八项固定列已停用。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>